<commit_message>
saved clean_names.xlsx without index
</commit_message>
<xml_diff>
--- a/clean_names.xlsx
+++ b/clean_names.xlsx
@@ -413,2511 +413,1761 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B251"/>
+  <dimension ref="A1:A251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>wolfgang frank fischer</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>SachIKO YOSHIkO YAMaMoTO</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>yuki hiroshi yamamoto</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>james robert rodriguez</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>tHoMAS RobeRT brOWN</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>márcia ana oliveira</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>angela angela colombo</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>mei lanh uang</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>catherine sylvie durand</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>MARCOS ANTÔNIO GOMES</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>mARíA CArmen CArMEN PéRez</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>LUIGI VINCENZO COLOMBO</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>carlos marcos oliveira</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>peter wolfgang fischer</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>peter klaus becker</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>fang juan wang</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>GIUSEPPE VINCENZO ROMANO</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>michael christopher rodriguez</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>vincenzo francesco marino</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>klaus michael wagner</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>isabel laura pérez</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>thomas robert martinez</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>alInE AlIne soUza</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>josé luis josé luis rodríguez</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>osamu hiroshi suzuki</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>jin yang liu</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>michael richard smith</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>marcOS JosÉ GoMES</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>keiko michiko ito</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>jing ping li</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>jessic alinda brown</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
-        <v>31</v>
-      </c>
-      <c r="B33" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>monika sabine schneider</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
-        <v>32</v>
-      </c>
-      <c r="B34" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>alain nicolas bernard</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
-        <v>33</v>
-      </c>
-      <c r="B35" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>klaus klaus wagner</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
-        <v>34</v>
-      </c>
-      <c r="B36" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>hans wolfgang weber</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
-        <v>35</v>
-      </c>
-      <c r="B37" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>frAnceScO viNCenzO rOsSI</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
-        <v>36</v>
-      </c>
-      <c r="B38" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>yoko yoshiko yamamoto</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
-        <v>37</v>
-      </c>
-      <c r="B39" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>david richard garcia</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
-        <v>38</v>
-      </c>
-      <c r="B40" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>christophe alain laurent</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
-        <v>39</v>
-      </c>
-      <c r="B41" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>michael john martinez</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
-        <v>40</v>
-      </c>
-      <c r="B42" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>maria ursula schulz</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
-        <v>41</v>
-      </c>
-      <c r="B43" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>josé luiz silva</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
-        <v>42</v>
-      </c>
-      <c r="B44" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>giovanni giuseppe marino</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
-        <v>43</v>
-      </c>
-      <c r="B45" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>klaus peter schneider</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
-        <v>44</v>
-      </c>
-      <c r="B46" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>yan yan zha g</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
-        <v>45</v>
-      </c>
-      <c r="B47" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>christian frank schmidt</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
-        <v>46</v>
-      </c>
-      <c r="B48" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>manuel francisco sánchez</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
-        <v>47</v>
-      </c>
-      <c r="B49" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>keiko yoko nakamura</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="n">
-        <v>48</v>
-      </c>
-      <c r="B50" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>ju nwei liu</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
-        <v>49</v>
-      </c>
-      <c r="B51" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>CHRISTIAN FRANK WEBER</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="n">
-        <v>50</v>
-      </c>
-      <c r="B52" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>petra ursula wagner</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="n">
-        <v>51</v>
-      </c>
-      <c r="B53" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>cArMelA GIOvannAR ICcI</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="n">
-        <v>52</v>
-      </c>
-      <c r="B54" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>antônio joão alves</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="n">
-        <v>53</v>
-      </c>
-      <c r="B55" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>fRANCISCo LuIz pEReiRA</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="n">
-        <v>54</v>
-      </c>
-      <c r="B56" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>fernanda maria oliveira</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="n">
-        <v>55</v>
-      </c>
-      <c r="B57" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>ling yan li</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="n">
-        <v>56</v>
-      </c>
-      <c r="B58" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>maría dolores maría dolores lópez</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="n">
-        <v>57</v>
-      </c>
-      <c r="B59" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>giuseppina giovanna marino</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="n">
-        <v>58</v>
-      </c>
-      <c r="B60" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>takashi akira nakamura</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="n">
-        <v>59</v>
-      </c>
-      <c r="B61" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>david richard martinez</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="n">
-        <v>60</v>
-      </c>
-      <c r="B62" t="inlineStr">
+      <c r="A62" t="inlineStr">
         <is>
           <t>christopher richard johnson</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="n">
-        <v>61</v>
-      </c>
-      <c r="B63" t="inlineStr">
+      <c r="A63" t="inlineStr">
         <is>
           <t>andreas wolfgang hoffmann</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="n">
-        <v>62</v>
-      </c>
-      <c r="B64" t="inlineStr">
+      <c r="A64" t="inlineStr">
         <is>
           <t>paulo paulo rodrigues</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="n">
-        <v>63</v>
-      </c>
-      <c r="B65" t="inlineStr">
+      <c r="A65" t="inlineStr">
         <is>
           <t>ursula petra schmidt</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="n">
-        <v>64</v>
-      </c>
-      <c r="B66" t="inlineStr">
+      <c r="A66" t="inlineStr">
         <is>
           <t>anna rosa greco</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="n">
-        <v>65</v>
-      </c>
-      <c r="B67" t="inlineStr">
+      <c r="A67" t="inlineStr">
         <is>
           <t>wililam thomas johnson</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="n">
-        <v>66</v>
-      </c>
-      <c r="B68" t="inlineStr">
+      <c r="A68" t="inlineStr">
         <is>
           <t>manuel josé sánchez</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="n">
-        <v>67</v>
-      </c>
-      <c r="B69" t="inlineStr">
+      <c r="A69" t="inlineStr">
         <is>
           <t>fernanda ana lima</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="n">
-        <v>68</v>
-      </c>
-      <c r="B70" t="inlineStr">
+      <c r="A70" t="inlineStr">
         <is>
           <t>CATHERINE MARTINE DUBOIS</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="n">
-        <v>69</v>
-      </c>
-      <c r="B71" t="inlineStr">
+      <c r="A71" t="inlineStr">
         <is>
           <t>giuseppe marior usso</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="n">
-        <v>70</v>
-      </c>
-      <c r="B72" t="inlineStr">
+      <c r="A72" t="inlineStr">
         <is>
           <t>marÍa DoLorEs TEresa garCiA</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="n">
-        <v>71</v>
-      </c>
-      <c r="B73" t="inlineStr">
+      <c r="A73" t="inlineStr">
         <is>
           <t>laura laura sánchez</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="n">
-        <v>72</v>
-      </c>
-      <c r="B74" t="inlineStr">
+      <c r="A74" t="inlineStr">
         <is>
           <t>rené NicOlAs tHOmaS</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="n">
-        <v>73</v>
-      </c>
-      <c r="B75" t="inlineStr">
+      <c r="A75" t="inlineStr">
         <is>
           <t>ANGElO AngElo mAriNO</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="n">
-        <v>74</v>
-      </c>
-      <c r="B76" t="inlineStr">
+      <c r="A76" t="inlineStr">
         <is>
           <t>lucia caterina russo</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="n">
-        <v>75</v>
-      </c>
-      <c r="B77" t="inlineStr">
+      <c r="A77" t="inlineStr">
         <is>
           <t>mary mary smith</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="n">
-        <v>76</v>
-      </c>
-      <c r="B78" t="inlineStr">
+      <c r="A78" t="inlineStr">
         <is>
           <t>fang ling liu</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="n">
-        <v>77</v>
-      </c>
-      <c r="B79" t="inlineStr">
+      <c r="A79" t="inlineStr">
         <is>
           <t>NAthalie moNIquE RoBeRt</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="n">
-        <v>78</v>
-      </c>
-      <c r="B80" t="inlineStr">
+      <c r="A80" t="inlineStr">
         <is>
           <t>rosa giuseppina rossi</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="n">
-        <v>79</v>
-      </c>
-      <c r="B81" t="inlineStr">
+      <c r="A81" t="inlineStr">
         <is>
           <t>yOShIko ToMoKO nAKAmuRA</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="n">
-        <v>80</v>
-      </c>
-      <c r="B82" t="inlineStr">
+      <c r="A82" t="inlineStr">
         <is>
           <t>antônio marcos silva</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="n">
-        <v>81</v>
-      </c>
-      <c r="B83" t="inlineStr">
+      <c r="A83" t="inlineStr">
         <is>
           <t>michiko yoshiko kobayashi</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="n">
-        <v>82</v>
-      </c>
-      <c r="B84" t="inlineStr">
+      <c r="A84" t="inlineStr">
         <is>
           <t>maria teresa ricci</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="n">
-        <v>83</v>
-      </c>
-      <c r="B85" t="inlineStr">
+      <c r="A85" t="inlineStr">
         <is>
           <t>ana maría carmen sánchez</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="n">
-        <v>84</v>
-      </c>
-      <c r="B86" t="inlineStr">
+      <c r="A86" t="inlineStr">
         <is>
           <t>ángel javier martínez</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="n">
-        <v>85</v>
-      </c>
-      <c r="B87" t="inlineStr">
+      <c r="A87" t="inlineStr">
         <is>
           <t>louis andré petit</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="n">
-        <v>86</v>
-      </c>
-      <c r="B88" t="inlineStr">
+      <c r="A88" t="inlineStr">
         <is>
           <t>fRaNk Frank fIschER</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="n">
-        <v>87</v>
-      </c>
-      <c r="B89" t="inlineStr">
+      <c r="A89" t="inlineStr">
         <is>
           <t>pierre michel durand</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="n">
-        <v>88</v>
-      </c>
-      <c r="B90" t="inlineStr">
+      <c r="A90" t="inlineStr">
         <is>
           <t>isabelle nathalie dubois</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="n">
-        <v>89</v>
-      </c>
-      <c r="B91" t="inlineStr">
+      <c r="A91" t="inlineStr">
         <is>
           <t>laUra MAria CARMEN roDrÍgUeZ</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="n">
-        <v>90</v>
-      </c>
-      <c r="B92" t="inlineStr">
+      <c r="A92" t="inlineStr">
         <is>
           <t>nicolas philippe robert</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="n">
-        <v>91</v>
-      </c>
-      <c r="B93" t="inlineStr">
+      <c r="A93" t="inlineStr">
         <is>
           <t>li jing wang</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="n">
-        <v>92</v>
-      </c>
-      <c r="B94" t="inlineStr">
+      <c r="A94" t="inlineStr">
         <is>
           <t>vincenzo vincenzo esposito</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="n">
-        <v>93</v>
-      </c>
-      <c r="B95" t="inlineStr">
+      <c r="A95" t="inlineStr">
         <is>
           <t>natHalie moNiqUe DuBoIs</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="n">
-        <v>94</v>
-      </c>
-      <c r="B96" t="inlineStr">
+      <c r="A96" t="inlineStr">
         <is>
           <t>sarah mary garcia</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="n">
-        <v>95</v>
-      </c>
-      <c r="B97" t="inlineStr">
+      <c r="A97" t="inlineStr">
         <is>
           <t>yan yan huang</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="n">
-        <v>96</v>
-      </c>
-      <c r="B98" t="inlineStr">
+      <c r="A98" t="inlineStr">
         <is>
           <t>adriana maria rodrigues</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="n">
-        <v>97</v>
-      </c>
-      <c r="B99" t="inlineStr">
+      <c r="A99" t="inlineStr">
         <is>
           <t>JAVIER DAVID LÓPEZ</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="n">
-        <v>98</v>
-      </c>
-      <c r="B100" t="inlineStr">
+      <c r="A100" t="inlineStr">
         <is>
           <t>carmela rosa greco</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="n">
-        <v>99</v>
-      </c>
-      <c r="B101" t="inlineStr">
+      <c r="A101" t="inlineStr">
         <is>
           <t>ping min zhao</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="n">
-        <v>100</v>
-      </c>
-      <c r="B102" t="inlineStr">
+      <c r="A102" t="inlineStr">
         <is>
           <t>yan fang li</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="n">
-        <v>101</v>
-      </c>
-      <c r="B103" t="inlineStr">
+      <c r="A103" t="inlineStr">
         <is>
           <t>david david fernández</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="n">
-        <v>102</v>
-      </c>
-      <c r="B104" t="inlineStr">
+      <c r="A104" t="inlineStr">
         <is>
           <t>giuseppe giuseppe esposito</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="n">
-        <v>103</v>
-      </c>
-      <c r="B105" t="inlineStr">
+      <c r="A105" t="inlineStr">
         <is>
           <t>josé david onzález</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="n">
-        <v>104</v>
-      </c>
-      <c r="B106" t="inlineStr">
+      <c r="A106" t="inlineStr">
         <is>
           <t>juan manuel rodríguez</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="n">
-        <v>105</v>
-      </c>
-      <c r="B107" t="inlineStr">
+      <c r="A107" t="inlineStr">
         <is>
           <t>sandrine sylvie moreau</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="n">
-        <v>106</v>
-      </c>
-      <c r="B108" t="inlineStr">
+      <c r="A108" t="inlineStr">
         <is>
           <t>fang lan wang</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="n">
-        <v>107</v>
-      </c>
-      <c r="B109" t="inlineStr">
+      <c r="A109" t="inlineStr">
         <is>
           <t>nathalie sylvie martin</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="n">
-        <v>108</v>
-      </c>
-      <c r="B110" t="inlineStr">
+      <c r="A110" t="inlineStr">
         <is>
           <t>rosa maria colombo</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="n">
-        <v>109</v>
-      </c>
-      <c r="B111" t="inlineStr">
+      <c r="A111" t="inlineStr">
         <is>
           <t>CatERina LUcia cOLOMBo</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="n">
-        <v>110</v>
-      </c>
-      <c r="B112" t="inlineStr">
+      <c r="A112" t="inlineStr">
         <is>
           <t>christophe nicolas richard</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="n">
-        <v>111</v>
-      </c>
-      <c r="B113" t="inlineStr">
+      <c r="A113" t="inlineStr">
         <is>
           <t>vincenzo salvatore russo</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="n">
-        <v>112</v>
-      </c>
-      <c r="B114" t="inlineStr">
+      <c r="A114" t="inlineStr">
         <is>
           <t>akira satoshi watanabe</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="n">
-        <v>113</v>
-      </c>
-      <c r="B115" t="inlineStr">
+      <c r="A115" t="inlineStr">
         <is>
           <t>JOSEPH THOMAS MILLRE</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="n">
-        <v>114</v>
-      </c>
-      <c r="B116" t="inlineStr">
+      <c r="A116" t="inlineStr">
         <is>
           <t>MARTINE ISABELLE RICHARD</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="n">
-        <v>115</v>
-      </c>
-      <c r="B117" t="inlineStr">
+      <c r="A117" t="inlineStr">
         <is>
           <t>luiz luiz oliveira</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="n">
-        <v>116</v>
-      </c>
-      <c r="B118" t="inlineStr">
+      <c r="A118" t="inlineStr">
         <is>
           <t>fraNcisco josé LuIs fERnÁndez</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="n">
-        <v>117</v>
-      </c>
-      <c r="B119" t="inlineStr">
+      <c r="A119" t="inlineStr">
         <is>
           <t>wililam wililam garcia</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="n">
-        <v>118</v>
-      </c>
-      <c r="B120" t="inlineStr">
+      <c r="A120" t="inlineStr">
         <is>
           <t>lucia angela rossi</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="n">
-        <v>119</v>
-      </c>
-      <c r="B121" t="inlineStr">
+      <c r="A121" t="inlineStr">
         <is>
           <t>ursula karin schulz</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="n">
-        <v>120</v>
-      </c>
-      <c r="B122" t="inlineStr">
+      <c r="A122" t="inlineStr">
         <is>
           <t>osamu hiroshi tanaka</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="n">
-        <v>121</v>
-      </c>
-      <c r="B123" t="inlineStr">
+      <c r="A123" t="inlineStr">
         <is>
           <t>yuki shinji ito</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="n">
-        <v>122</v>
-      </c>
-      <c r="B124" t="inlineStr">
+      <c r="A124" t="inlineStr">
         <is>
           <t>wolfgang andreas weber</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="n">
-        <v>123</v>
-      </c>
-      <c r="B125" t="inlineStr">
+      <c r="A125" t="inlineStr">
         <is>
           <t>pietro giovanni esposito</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="n">
-        <v>124</v>
-      </c>
-      <c r="B126" t="inlineStr">
+      <c r="A126" t="inlineStr">
         <is>
           <t>teresa maría carmen martínez</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="n">
-        <v>125</v>
-      </c>
-      <c r="B127" t="inlineStr">
+      <c r="A127" t="inlineStr">
         <is>
           <t>ANgELA CARMELA GRECO</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="n">
-        <v>126</v>
-      </c>
-      <c r="B128" t="inlineStr">
+      <c r="A128" t="inlineStr">
         <is>
           <t>christian klaus fischer</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="n">
-        <v>127</v>
-      </c>
-      <c r="B129" t="inlineStr">
+      <c r="A129" t="inlineStr">
         <is>
           <t>lucas luiz gomes</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="n">
-        <v>128</v>
-      </c>
-      <c r="B130" t="inlineStr">
+      <c r="A130" t="inlineStr">
         <is>
           <t>pietro angelo russo</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" t="n">
-        <v>129</v>
-      </c>
-      <c r="B131" t="inlineStr">
+      <c r="A131" t="inlineStr">
         <is>
           <t>JOSÉ ANTÔNIO L IMA</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" t="n">
-        <v>130</v>
-      </c>
-      <c r="B132" t="inlineStr">
+      <c r="A132" t="inlineStr">
         <is>
           <t>laura maría lópez</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="A133" t="n">
-        <v>131</v>
-      </c>
-      <c r="B133" t="inlineStr">
+      <c r="A133" t="inlineStr">
         <is>
           <t>michael klaus schmidt</t>
         </is>
       </c>
     </row>
     <row r="134">
-      <c r="A134" t="n">
-        <v>132</v>
-      </c>
-      <c r="B134" t="inlineStr">
+      <c r="A134" t="inlineStr">
         <is>
           <t>hiroko yoko tanaka</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="A135" t="n">
-        <v>133</v>
-      </c>
-      <c r="B135" t="inlineStr">
+      <c r="A135" t="inlineStr">
         <is>
           <t>MIN LINGZ HANG</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" t="n">
-        <v>134</v>
-      </c>
-      <c r="B136" t="inlineStr">
+      <c r="A136" t="inlineStr">
         <is>
           <t>giovanna carmela romano</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" t="n">
-        <v>135</v>
-      </c>
-      <c r="B137" t="inlineStr">
+      <c r="A137" t="inlineStr">
         <is>
           <t>monique sandrine robert</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="A138" t="n">
-        <v>136</v>
-      </c>
-      <c r="B138" t="inlineStr">
+      <c r="A138" t="inlineStr">
         <is>
           <t>gang lei zhou</t>
         </is>
       </c>
     </row>
     <row r="139">
-      <c r="A139" t="n">
-        <v>137</v>
-      </c>
-      <c r="B139" t="inlineStr">
+      <c r="A139" t="inlineStr">
         <is>
           <t>ANToNio AnTONio gÓMez</t>
         </is>
       </c>
     </row>
     <row r="140">
-      <c r="A140" t="n">
-        <v>138</v>
-      </c>
-      <c r="B140" t="inlineStr">
+      <c r="A140" t="inlineStr">
         <is>
           <t>marcos josé silva</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" t="n">
-        <v>139</v>
-      </c>
-      <c r="B141" t="inlineStr">
+      <c r="A141" t="inlineStr">
         <is>
           <t>jie hao yang</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="A142" t="n">
-        <v>140</v>
-      </c>
-      <c r="B142" t="inlineStr">
+      <c r="A142" t="inlineStr">
         <is>
           <t>ping fang wu</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="A143" t="n">
-        <v>141</v>
-      </c>
-      <c r="B143" t="inlineStr">
+      <c r="A143" t="inlineStr">
         <is>
           <t>mei lan wu</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" t="n">
-        <v>142</v>
-      </c>
-      <c r="B144" t="inlineStr">
+      <c r="A144" t="inlineStr">
         <is>
           <t>alain jea nthomas</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="A145" t="n">
-        <v>143</v>
-      </c>
-      <c r="B145" t="inlineStr">
+      <c r="A145" t="inlineStr">
         <is>
           <t>sandrine sandrine durand</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" t="n">
-        <v>144</v>
-      </c>
-      <c r="B146" t="inlineStr">
+      <c r="A146" t="inlineStr">
         <is>
           <t>maría maría carmen gómez</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" t="n">
-        <v>145</v>
-      </c>
-      <c r="B147" t="inlineStr">
+      <c r="A147" t="inlineStr">
         <is>
           <t>michael michael schmidt</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="n">
-        <v>146</v>
-      </c>
-      <c r="B148" t="inlineStr">
+      <c r="A148" t="inlineStr">
         <is>
           <t>lucas marcos rodrigues</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="n">
-        <v>147</v>
-      </c>
-      <c r="B149" t="inlineStr">
+      <c r="A149" t="inlineStr">
         <is>
           <t>lan fang zhao</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="n">
-        <v>148</v>
-      </c>
-      <c r="B150" t="inlineStr">
+      <c r="A150" t="inlineStr">
         <is>
           <t>jennifer susan jones</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="n">
-        <v>149</v>
-      </c>
-      <c r="B151" t="inlineStr">
+      <c r="A151" t="inlineStr">
         <is>
           <t>ping yan yang</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="n">
-        <v>150</v>
-      </c>
-      <c r="B152" t="inlineStr">
+      <c r="A152" t="inlineStr">
         <is>
           <t>francesco mario ferrari</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="n">
-        <v>151</v>
-      </c>
-      <c r="B153" t="inlineStr">
+      <c r="A153" t="inlineStr">
         <is>
           <t>christopher christopher johnson</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="n">
-        <v>152</v>
-      </c>
-      <c r="B154" t="inlineStr">
+      <c r="A154" t="inlineStr">
         <is>
           <t>HANS WOLFGANG BECKeR</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="n">
-        <v>153</v>
-      </c>
-      <c r="B155" t="inlineStr">
+      <c r="A155" t="inlineStr">
         <is>
           <t>jeSsIca sUSan JoNes</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="n">
-        <v>154</v>
-      </c>
-      <c r="B156" t="inlineStr">
+      <c r="A156" t="inlineStr">
         <is>
           <t>MASAKO HIROKO KOBAYASHI</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="A157" t="n">
-        <v>155</v>
-      </c>
-      <c r="B157" t="inlineStr">
+      <c r="A157" t="inlineStr">
         <is>
           <t>FRaNcisCo anTÔnio silvA</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="n">
-        <v>156</v>
-      </c>
-      <c r="B158" t="inlineStr">
+      <c r="A158" t="inlineStr">
         <is>
           <t>danile francisco martin</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="n">
-        <v>157</v>
-      </c>
-      <c r="B159" t="inlineStr">
+      <c r="A159" t="inlineStr">
         <is>
           <t>isabelle catherine martin</t>
         </is>
       </c>
     </row>
     <row r="160">
-      <c r="A160" t="n">
-        <v>158</v>
-      </c>
-      <c r="B160" t="inlineStr">
+      <c r="A160" t="inlineStr">
         <is>
           <t>miCHIko YosHiKo YamAmOTO</t>
         </is>
       </c>
     </row>
     <row r="161">
-      <c r="A161" t="n">
-        <v>159</v>
-      </c>
-      <c r="B161" t="inlineStr">
+      <c r="A161" t="inlineStr">
         <is>
           <t>jie lei li</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="A162" t="n">
-        <v>160</v>
-      </c>
-      <c r="B162" t="inlineStr">
+      <c r="A162" t="inlineStr">
         <is>
           <t>juliana aline silva</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="A163" t="n">
-        <v>161</v>
-      </c>
-      <c r="B163" t="inlineStr">
+      <c r="A163" t="inlineStr">
         <is>
           <t>rené louis dubois</t>
         </is>
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="n">
-        <v>162</v>
-      </c>
-      <c r="B164" t="inlineStr">
+      <c r="A164" t="inlineStr">
         <is>
           <t>ALINE ALINE SANTOS</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" t="n">
-        <v>163</v>
-      </c>
-      <c r="B165" t="inlineStr">
+      <c r="A165" t="inlineStr">
         <is>
           <t>hiroko michiko ito</t>
         </is>
       </c>
     </row>
     <row r="166">
-      <c r="A166" t="n">
-        <v>164</v>
-      </c>
-      <c r="B166" t="inlineStr">
+      <c r="A166" t="inlineStr">
         <is>
           <t>stefan stefan müller</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="A167" t="n">
-        <v>165</v>
-      </c>
-      <c r="B167" t="inlineStr">
+      <c r="A167" t="inlineStr">
         <is>
           <t>fernanda maria lima</t>
         </is>
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="n">
-        <v>166</v>
-      </c>
-      <c r="B168" t="inlineStr">
+      <c r="A168" t="inlineStr">
         <is>
           <t>christian frank müller</t>
         </is>
       </c>
     </row>
     <row r="169">
-      <c r="A169" t="n">
-        <v>167</v>
-      </c>
-      <c r="B169" t="inlineStr">
+      <c r="A169" t="inlineStr">
         <is>
           <t>Yuki hIrOsHI WATAnaBe</t>
         </is>
       </c>
     </row>
     <row r="170">
-      <c r="A170" t="n">
-        <v>168</v>
-      </c>
-      <c r="B170" t="inlineStr">
+      <c r="A170" t="inlineStr">
         <is>
           <t>petra ursula fischer</t>
         </is>
       </c>
     </row>
     <row r="171">
-      <c r="A171" t="n">
-        <v>169</v>
-      </c>
-      <c r="B171" t="inlineStr">
+      <c r="A171" t="inlineStr">
         <is>
           <t>robert john garcia</t>
         </is>
       </c>
     </row>
     <row r="172">
-      <c r="A172" t="n">
-        <v>170</v>
-      </c>
-      <c r="B172" t="inlineStr">
+      <c r="A172" t="inlineStr">
         <is>
           <t>mary susan jones</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" t="n">
-        <v>171</v>
-      </c>
-      <c r="B173" t="inlineStr">
+      <c r="A173" t="inlineStr">
         <is>
           <t>richard joseph williasm</t>
         </is>
       </c>
     </row>
     <row r="174">
-      <c r="A174" t="n">
-        <v>172</v>
-      </c>
-      <c r="B174" t="inlineStr">
+      <c r="A174" t="inlineStr">
         <is>
           <t>FRANCISCO FRANCISCO MARTIN</t>
         </is>
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="n">
-        <v>173</v>
-      </c>
-      <c r="B175" t="inlineStr">
+      <c r="A175" t="inlineStr">
         <is>
           <t>fang jun liu</t>
         </is>
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="n">
-        <v>174</v>
-      </c>
-      <c r="B176" t="inlineStr">
+      <c r="A176" t="inlineStr">
         <is>
           <t>aline francisca santos</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="n">
-        <v>175</v>
-      </c>
-      <c r="B177" t="inlineStr">
+      <c r="A177" t="inlineStr">
         <is>
           <t>salvatore giovanni rossi</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="n">
-        <v>176</v>
-      </c>
-      <c r="B178" t="inlineStr">
+      <c r="A178" t="inlineStr">
         <is>
           <t>monique marie thomas</t>
         </is>
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="n">
-        <v>177</v>
-      </c>
-      <c r="B179" t="inlineStr">
+      <c r="A179" t="inlineStr">
         <is>
           <t>antônia antônia oliveira</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="n">
-        <v>178</v>
-      </c>
-      <c r="B180" t="inlineStr">
+      <c r="A180" t="inlineStr">
         <is>
           <t>cARMELa lUCia ferRARI</t>
         </is>
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="n">
-        <v>179</v>
-      </c>
-      <c r="B181" t="inlineStr">
+      <c r="A181" t="inlineStr">
         <is>
           <t>juliana antônia ferreira</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="A182" t="n">
-        <v>180</v>
-      </c>
-      <c r="B182" t="inlineStr">
+      <c r="A182" t="inlineStr">
         <is>
           <t>klaus wolfgang meyer</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="n">
-        <v>181</v>
-      </c>
-      <c r="B183" t="inlineStr">
+      <c r="A183" t="inlineStr">
         <is>
           <t>yan ping huang</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="n">
-        <v>182</v>
-      </c>
-      <c r="B184" t="inlineStr">
+      <c r="A184" t="inlineStr">
         <is>
           <t>josé luis danile fernández</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" t="n">
-        <v>183</v>
-      </c>
-      <c r="B185" t="inlineStr">
+      <c r="A185" t="inlineStr">
         <is>
           <t>rené christophe robert</t>
         </is>
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="n">
-        <v>184</v>
-      </c>
-      <c r="B186" t="inlineStr">
+      <c r="A186" t="inlineStr">
         <is>
           <t>lucia angela colombo</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="n">
-        <v>185</v>
-      </c>
-      <c r="B187" t="inlineStr">
+      <c r="A187" t="inlineStr">
         <is>
           <t>maria sabine weber</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="n">
-        <v>186</v>
-      </c>
-      <c r="B188" t="inlineStr">
+      <c r="A188" t="inlineStr">
         <is>
           <t>juliana maria ferreira</t>
         </is>
       </c>
     </row>
     <row r="189">
-      <c r="A189" t="n">
-        <v>187</v>
-      </c>
-      <c r="B189" t="inlineStr">
+      <c r="A189" t="inlineStr">
         <is>
           <t>renate maria hoffmann</t>
         </is>
       </c>
     </row>
     <row r="190">
-      <c r="A190" t="n">
-        <v>188</v>
-      </c>
-      <c r="B190" t="inlineStr">
+      <c r="A190" t="inlineStr">
         <is>
           <t>ana antônia gomes</t>
         </is>
       </c>
     </row>
     <row r="191">
-      <c r="A191" t="n">
-        <v>189</v>
-      </c>
-      <c r="B191" t="inlineStr">
+      <c r="A191" t="inlineStr">
         <is>
           <t>hao lei li</t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="A192" t="n">
-        <v>190</v>
-      </c>
-      <c r="B192" t="inlineStr">
+      <c r="A192" t="inlineStr">
         <is>
           <t>KENJi toRu WATaNABe</t>
         </is>
       </c>
     </row>
     <row r="193">
-      <c r="A193" t="n">
-        <v>191</v>
-      </c>
-      <c r="B193" t="inlineStr">
+      <c r="A193" t="inlineStr">
         <is>
           <t>françoise martine thomas</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" t="n">
-        <v>192</v>
-      </c>
-      <c r="B194" t="inlineStr">
+      <c r="A194" t="inlineStr">
         <is>
           <t>toru yuki kobayashi</t>
         </is>
       </c>
     </row>
     <row r="195">
-      <c r="A195" t="n">
-        <v>193</v>
-      </c>
-      <c r="B195" t="inlineStr">
+      <c r="A195" t="inlineStr">
         <is>
           <t>andreas peter schneider</t>
         </is>
       </c>
     </row>
     <row r="196">
-      <c r="A196" t="n">
-        <v>194</v>
-      </c>
-      <c r="B196" t="inlineStr">
+      <c r="A196" t="inlineStr">
         <is>
           <t>akiko yoshiko suzuki</t>
         </is>
       </c>
     </row>
     <row r="197">
-      <c r="A197" t="n">
-        <v>195</v>
-      </c>
-      <c r="B197" t="inlineStr">
+      <c r="A197" t="inlineStr">
         <is>
           <t>yang ju nyang</t>
         </is>
       </c>
     </row>
     <row r="198">
-      <c r="A198" t="n">
-        <v>196</v>
-      </c>
-      <c r="B198" t="inlineStr">
+      <c r="A198" t="inlineStr">
         <is>
           <t>angelo pietro bianchi</t>
         </is>
       </c>
     </row>
     <row r="199">
-      <c r="A199" t="n">
-        <v>197</v>
-      </c>
-      <c r="B199" t="inlineStr">
+      <c r="A199" t="inlineStr">
         <is>
           <t>min lan wang</t>
         </is>
       </c>
     </row>
     <row r="200">
-      <c r="A200" t="n">
-        <v>198</v>
-      </c>
-      <c r="B200" t="inlineStr">
+      <c r="A200" t="inlineStr">
         <is>
           <t>juliana fernanda silva</t>
         </is>
       </c>
     </row>
     <row r="201">
-      <c r="A201" t="n">
-        <v>199</v>
-      </c>
-      <c r="B201" t="inlineStr">
+      <c r="A201" t="inlineStr">
         <is>
           <t>angelo giuseppe ricci</t>
         </is>
       </c>
     </row>
     <row r="202">
-      <c r="A202" t="n">
-        <v>200</v>
-      </c>
-      <c r="B202" t="inlineStr">
+      <c r="A202" t="inlineStr">
         <is>
           <t>alain andré robert</t>
         </is>
       </c>
     </row>
     <row r="203">
-      <c r="A203" t="n">
-        <v>201</v>
-      </c>
-      <c r="B203" t="inlineStr">
+      <c r="A203" t="inlineStr">
         <is>
           <t>maria rosa ferrari</t>
         </is>
       </c>
     </row>
     <row r="204">
-      <c r="A204" t="n">
-        <v>202</v>
-      </c>
-      <c r="B204" t="inlineStr">
+      <c r="A204" t="inlineStr">
         <is>
           <t>ANDRÉ RENÉ RICHARD</t>
         </is>
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="n">
-        <v>203</v>
-      </c>
-      <c r="B205" t="inlineStr">
+      <c r="A205" t="inlineStr">
         <is>
           <t>akira kenji kobayashi</t>
         </is>
       </c>
     </row>
     <row r="206">
-      <c r="A206" t="n">
-        <v>204</v>
-      </c>
-      <c r="B206" t="inlineStr">
+      <c r="A206" t="inlineStr">
         <is>
           <t>joseph thomas martinez</t>
         </is>
       </c>
     </row>
     <row r="207">
-      <c r="A207" t="n">
-        <v>205</v>
-      </c>
-      <c r="B207" t="inlineStr">
+      <c r="A207" t="inlineStr">
         <is>
           <t>ISABEL TERESA LÓPEZ</t>
         </is>
       </c>
     </row>
     <row r="208">
-      <c r="A208" t="n">
-        <v>206</v>
-      </c>
-      <c r="B208" t="inlineStr">
+      <c r="A208" t="inlineStr">
         <is>
           <t>li yan chen</t>
         </is>
       </c>
     </row>
     <row r="209">
-      <c r="A209" t="n">
-        <v>207</v>
-      </c>
-      <c r="B209" t="inlineStr">
+      <c r="A209" t="inlineStr">
         <is>
           <t>nicolas jean laurent</t>
         </is>
       </c>
     </row>
     <row r="210">
-      <c r="A210" t="n">
-        <v>208</v>
-      </c>
-      <c r="B210" t="inlineStr">
+      <c r="A210" t="inlineStr">
         <is>
           <t>HelgA Sabine MeyER</t>
         </is>
       </c>
     </row>
     <row r="211">
-      <c r="A211" t="n">
-        <v>209</v>
-      </c>
-      <c r="B211" t="inlineStr">
+      <c r="A211" t="inlineStr">
         <is>
           <t>rosa teresa ricci</t>
         </is>
       </c>
     </row>
     <row r="212">
-      <c r="A212" t="n">
-        <v>210</v>
-      </c>
-      <c r="B212" t="inlineStr">
+      <c r="A212" t="inlineStr">
         <is>
           <t>min min wu</t>
         </is>
       </c>
     </row>
     <row r="213">
-      <c r="A213" t="n">
-        <v>211</v>
-      </c>
-      <c r="B213" t="inlineStr">
+      <c r="A213" t="inlineStr">
         <is>
           <t>yang qiang zhao</t>
         </is>
       </c>
     </row>
     <row r="214">
-      <c r="A214" t="n">
-        <v>212</v>
-      </c>
-      <c r="B214" t="inlineStr">
+      <c r="A214" t="inlineStr">
         <is>
           <t>josé luis josé luis fernández</t>
         </is>
       </c>
     </row>
     <row r="215">
-      <c r="A215" t="n">
-        <v>213</v>
-      </c>
-      <c r="B215" t="inlineStr">
+      <c r="A215" t="inlineStr">
         <is>
           <t>hiroshi satoshi tanaka</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" t="n">
-        <v>214</v>
-      </c>
-      <c r="B216" t="inlineStr">
+      <c r="A216" t="inlineStr">
         <is>
           <t>THOMAS THOMAS SCHNEIDER</t>
         </is>
       </c>
     </row>
     <row r="217">
-      <c r="A217" t="n">
-        <v>215</v>
-      </c>
-      <c r="B217" t="inlineStr">
+      <c r="A217" t="inlineStr">
         <is>
           <t>nathalie sandrine moreau</t>
         </is>
       </c>
     </row>
     <row r="218">
-      <c r="A218" t="n">
-        <v>216</v>
-      </c>
-      <c r="B218" t="inlineStr">
+      <c r="A218" t="inlineStr">
         <is>
           <t>hans hans wagner</t>
         </is>
       </c>
     </row>
     <row r="219">
-      <c r="A219" t="n">
-        <v>217</v>
-      </c>
-      <c r="B219" t="inlineStr">
+      <c r="A219" t="inlineStr">
         <is>
           <t>sarah mary millre</t>
         </is>
       </c>
     </row>
     <row r="220">
-      <c r="A220" t="n">
-        <v>218</v>
-      </c>
-      <c r="B220" t="inlineStr">
+      <c r="A220" t="inlineStr">
         <is>
           <t>josefa maría pilar pérez</t>
         </is>
       </c>
     </row>
     <row r="221">
-      <c r="A221" t="n">
-        <v>219</v>
-      </c>
-      <c r="B221" t="inlineStr">
+      <c r="A221" t="inlineStr">
         <is>
           <t>márcia juliana pereira</t>
         </is>
       </c>
     </row>
     <row r="222">
-      <c r="A222" t="n">
-        <v>220</v>
-      </c>
-      <c r="B222" t="inlineStr">
+      <c r="A222" t="inlineStr">
         <is>
           <t>marcos antônio oliveira</t>
         </is>
       </c>
     </row>
     <row r="223">
-      <c r="A223" t="n">
-        <v>221</v>
-      </c>
-      <c r="B223" t="inlineStr">
+      <c r="A223" t="inlineStr">
         <is>
           <t>masako yoko ito</t>
         </is>
       </c>
     </row>
     <row r="224">
-      <c r="A224" t="n">
-        <v>222</v>
-      </c>
-      <c r="B224" t="inlineStr">
+      <c r="A224" t="inlineStr">
         <is>
           <t>wolfgang michael hoffmann</t>
         </is>
       </c>
     </row>
     <row r="225">
-      <c r="A225" t="n">
-        <v>223</v>
-      </c>
-      <c r="B225" t="inlineStr">
+      <c r="A225" t="inlineStr">
         <is>
           <t>nathalie françoise robert</t>
         </is>
       </c>
     </row>
     <row r="226">
-      <c r="A226" t="n">
-        <v>224</v>
-      </c>
-      <c r="B226" t="inlineStr">
+      <c r="A226" t="inlineStr">
         <is>
           <t>francisca adriana lima</t>
         </is>
       </c>
     </row>
     <row r="227">
-      <c r="A227" t="n">
-        <v>225</v>
-      </c>
-      <c r="B227" t="inlineStr">
+      <c r="A227" t="inlineStr">
         <is>
           <t>ANGELA CARMELA BIANCHI</t>
         </is>
       </c>
     </row>
     <row r="228">
-      <c r="A228" t="n">
-        <v>226</v>
-      </c>
-      <c r="B228" t="inlineStr">
+      <c r="A228" t="inlineStr">
         <is>
           <t>FANG MIn LI</t>
         </is>
       </c>
     </row>
     <row r="229">
-      <c r="A229" t="n">
-        <v>227</v>
-      </c>
-      <c r="B229" t="inlineStr">
+      <c r="A229" t="inlineStr">
         <is>
           <t>patrícia aline ferreira</t>
         </is>
       </c>
     </row>
     <row r="230">
-      <c r="A230" t="n">
-        <v>228</v>
-      </c>
-      <c r="B230" t="inlineStr">
+      <c r="A230" t="inlineStr">
         <is>
           <t>angela maria romano</t>
         </is>
       </c>
     </row>
     <row r="231">
-      <c r="A231" t="n">
-        <v>229</v>
-      </c>
-      <c r="B231" t="inlineStr">
+      <c r="A231" t="inlineStr">
         <is>
           <t>alain christophe petit</t>
         </is>
       </c>
     </row>
     <row r="232">
-      <c r="A232" t="n">
-        <v>230</v>
-      </c>
-      <c r="B232" t="inlineStr">
+      <c r="A232" t="inlineStr">
         <is>
           <t>barbara jessica rodriguez</t>
         </is>
       </c>
     </row>
     <row r="233">
-      <c r="A233" t="n">
-        <v>231</v>
-      </c>
-      <c r="B233" t="inlineStr">
+      <c r="A233" t="inlineStr">
         <is>
           <t>josé antonio gómez</t>
         </is>
       </c>
     </row>
     <row r="234">
-      <c r="A234" t="n">
-        <v>232</v>
-      </c>
-      <c r="B234" t="inlineStr">
+      <c r="A234" t="inlineStr">
         <is>
           <t>hAo qianG zhaO</t>
         </is>
       </c>
     </row>
     <row r="235">
-      <c r="A235" t="n">
-        <v>233</v>
-      </c>
-      <c r="B235" t="inlineStr">
+      <c r="A235" t="inlineStr">
         <is>
           <t>tomoko tomoko kato</t>
         </is>
       </c>
     </row>
     <row r="236">
-      <c r="A236" t="n">
-        <v>234</v>
-      </c>
-      <c r="B236" t="inlineStr">
+      <c r="A236" t="inlineStr">
         <is>
           <t>linda jessica brown</t>
         </is>
       </c>
     </row>
     <row r="237">
-      <c r="A237" t="n">
-        <v>235</v>
-      </c>
-      <c r="B237" t="inlineStr">
+      <c r="A237" t="inlineStr">
         <is>
           <t>sandrin emonique moreau</t>
         </is>
       </c>
     </row>
     <row r="238">
-      <c r="A238" t="n">
-        <v>236</v>
-      </c>
-      <c r="B238" t="inlineStr">
+      <c r="A238" t="inlineStr">
         <is>
           <t>NAOKO MICHIKO NAKAmURA</t>
         </is>
       </c>
     </row>
     <row r="239">
-      <c r="A239" t="n">
-        <v>237</v>
-      </c>
-      <c r="B239" t="inlineStr">
+      <c r="A239" t="inlineStr">
         <is>
           <t>maria antônia gomes</t>
         </is>
       </c>
     </row>
     <row r="240">
-      <c r="A240" t="n">
-        <v>238</v>
-      </c>
-      <c r="B240" t="inlineStr">
+      <c r="A240" t="inlineStr">
         <is>
           <t>patrícia adriana alves</t>
         </is>
       </c>
     </row>
     <row r="241">
-      <c r="A241" t="n">
-        <v>239</v>
-      </c>
-      <c r="B241" t="inlineStr">
+      <c r="A241" t="inlineStr">
         <is>
           <t>SANDRINE MONIQuE LAURENT</t>
         </is>
       </c>
     </row>
     <row r="242">
-      <c r="A242" t="n">
-        <v>240</v>
-      </c>
-      <c r="B242" t="inlineStr">
+      <c r="A242" t="inlineStr">
         <is>
           <t>nicolas michel thomas</t>
         </is>
       </c>
     </row>
     <row r="243">
-      <c r="A243" t="n">
-        <v>241</v>
-      </c>
-      <c r="B243" t="inlineStr">
+      <c r="A243" t="inlineStr">
         <is>
           <t>andreas klaus becker</t>
         </is>
       </c>
     </row>
     <row r="244">
-      <c r="A244" t="n">
-        <v>242</v>
-      </c>
-      <c r="B244" t="inlineStr">
+      <c r="A244" t="inlineStr">
         <is>
           <t>stefan stefan meyer</t>
         </is>
       </c>
     </row>
     <row r="245">
-      <c r="A245" t="n">
-        <v>243</v>
-      </c>
-      <c r="B245" t="inlineStr">
+      <c r="A245" t="inlineStr">
         <is>
           <t>linda sarah brown</t>
         </is>
       </c>
     </row>
     <row r="246">
-      <c r="A246" t="n">
-        <v>244</v>
-      </c>
-      <c r="B246" t="inlineStr">
+      <c r="A246" t="inlineStr">
         <is>
           <t>lucas paulo lima</t>
         </is>
       </c>
     </row>
     <row r="247">
-      <c r="A247" t="n">
-        <v>245</v>
-      </c>
-      <c r="B247" t="inlineStr">
+      <c r="A247" t="inlineStr">
         <is>
           <t>andré rené moreau</t>
         </is>
       </c>
     </row>
     <row r="248">
-      <c r="A248" t="n">
-        <v>246</v>
-      </c>
-      <c r="B248" t="inlineStr">
+      <c r="A248" t="inlineStr">
         <is>
           <t>sachiko tomoko sato</t>
         </is>
       </c>
     </row>
     <row r="249">
-      <c r="A249" t="n">
-        <v>247</v>
-      </c>
-      <c r="B249" t="inlineStr">
+      <c r="A249" t="inlineStr">
         <is>
           <t>lan mei li</t>
         </is>
       </c>
     </row>
     <row r="250">
-      <c r="A250" t="n">
-        <v>248</v>
-      </c>
-      <c r="B250" t="inlineStr">
+      <c r="A250" t="inlineStr">
         <is>
           <t>isabel teresa rodríguez</t>
         </is>
       </c>
     </row>
     <row r="251">
-      <c r="A251" t="n">
-        <v>249</v>
-      </c>
-      <c r="B251" t="inlineStr">
+      <c r="A251" t="inlineStr">
         <is>
           <t>sylvie françoise robert</t>
         </is>

</xml_diff>